<commit_message>
102 Game week 14 update
</commit_message>
<xml_diff>
--- a/data/latest_data.xlsx
+++ b/data/latest_data.xlsx
@@ -15,14 +15,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="IM5lxP9hLCN1ssUYGypgzn83w03NwZfLY2qp78uklxw="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="Q8pwG3tm1Blk2/1BcBGXSUPrEhsW2sZE0Hv4sE5tRhM="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="181">
   <si>
     <t>MARLOW DUKES 2025</t>
   </si>
@@ -234,9 +234,6 @@
     <t>GOBBY</t>
   </si>
   <si>
-    <t>BRUCE</t>
-  </si>
-  <si>
     <t>DUNCAN</t>
   </si>
   <si>
@@ -246,13 +243,16 @@
     <t>SONES</t>
   </si>
   <si>
+    <t>BRUCE</t>
+  </si>
+  <si>
     <t>DWARF</t>
   </si>
   <si>
-    <t>BANKSY</t>
+    <t>ARTIST</t>
   </si>
   <si>
-    <t>ARTIST</t>
+    <t>BANKSY</t>
   </si>
   <si>
     <t>GUEST 2</t>
@@ -345,6 +345,9 @@
     <t xml:space="preserve"> 6-4</t>
   </si>
   <si>
+    <t xml:space="preserve"> 1-1</t>
+  </si>
+  <si>
     <t>P</t>
   </si>
   <si>
@@ -370,9 +373,6 @@
   </si>
   <si>
     <t>MAMAS</t>
-  </si>
-  <si>
-    <t>DOM</t>
   </si>
   <si>
     <t>MICK</t>
@@ -550,6 +550,12 @@
   </si>
   <si>
     <t>Flo</t>
+  </si>
+  <si>
+    <t>Posh v Preston</t>
+  </si>
+  <si>
+    <t>Drew 1-1</t>
   </si>
   <si>
     <t>Moo</t>
@@ -786,7 +792,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="68">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -939,9 +945,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -1664,7 +1667,9 @@
       <c r="N5" s="16">
         <v>2.0</v>
       </c>
-      <c r="O5" s="16"/>
+      <c r="O5" s="17">
+        <v>0.0</v>
+      </c>
       <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
@@ -1705,7 +1710,7 @@
       </c>
       <c r="AZ5" s="5">
         <f t="shared" ref="AZ5:AZ40" si="1">COUNT(B5:AX5)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="BA5" s="5">
         <f t="shared" ref="BA5:BA40" si="2">COUNTIF($B5:$AX5, "&gt;=1")</f>
@@ -1713,7 +1718,7 @@
       </c>
       <c r="BB5" s="5">
         <f t="shared" ref="BB5:BB40" si="3">COUNTIF($B5:$AX5, "0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC5" s="5">
         <f t="shared" ref="BC5:BC40" si="4">COUNTIF($B5:$AX5, "&lt;0")</f>
@@ -1721,7 +1726,7 @@
       </c>
       <c r="BD5" s="5">
         <f t="shared" ref="BD5:BD40" si="5">SUM(BA5*3)+BB5</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="BE5" s="5">
         <f t="shared" ref="BE5:BE40" si="6">SUM(B5:AX5)</f>
@@ -1729,7 +1734,7 @@
       </c>
       <c r="BF5" s="20">
         <f t="shared" ref="BF5:BF40" si="7">SUM(BA5*3+BB5*1)/SUM(AZ5*3)</f>
-        <v>0.6666666667</v>
+        <v>0.641025641</v>
       </c>
       <c r="BG5" s="20"/>
     </row>
@@ -1770,7 +1775,9 @@
       <c r="N6" s="23">
         <v>2.0</v>
       </c>
-      <c r="O6" s="23"/>
+      <c r="O6" s="23">
+        <v>0.0</v>
+      </c>
       <c r="P6" s="23"/>
       <c r="Q6" s="23"/>
       <c r="R6" s="23"/>
@@ -1811,7 +1818,7 @@
       </c>
       <c r="AZ6" s="5">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BA6" s="5">
         <f t="shared" si="2"/>
@@ -1819,7 +1826,7 @@
       </c>
       <c r="BB6" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC6" s="5">
         <f t="shared" si="4"/>
@@ -1827,7 +1834,7 @@
       </c>
       <c r="BD6" s="5">
         <f t="shared" si="5"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="BE6" s="5">
         <f t="shared" si="6"/>
@@ -1835,7 +1842,7 @@
       </c>
       <c r="BF6" s="20">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.5757575758</v>
       </c>
       <c r="BG6" s="20"/>
     </row>
@@ -1880,7 +1887,9 @@
       <c r="N7" s="28">
         <v>-2.0</v>
       </c>
-      <c r="O7" s="28"/>
+      <c r="O7" s="29">
+        <v>0.0</v>
+      </c>
       <c r="P7" s="28"/>
       <c r="Q7" s="28"/>
       <c r="R7" s="28"/>
@@ -1921,7 +1930,7 @@
       </c>
       <c r="AZ7" s="5">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="BA7" s="5">
         <f t="shared" si="2"/>
@@ -1929,7 +1938,7 @@
       </c>
       <c r="BB7" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC7" s="5">
         <f t="shared" si="4"/>
@@ -1937,7 +1946,7 @@
       </c>
       <c r="BD7" s="5">
         <f t="shared" si="5"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="BE7" s="5">
         <f t="shared" si="6"/>
@@ -1945,7 +1954,7 @@
       </c>
       <c r="BF7" s="20">
         <f t="shared" si="7"/>
-        <v>0.5</v>
+        <v>0.4871794872</v>
       </c>
       <c r="BG7" s="20"/>
     </row>
@@ -1986,7 +1995,9 @@
       <c r="N8" s="16">
         <v>-2.0</v>
       </c>
-      <c r="O8" s="16"/>
+      <c r="O8" s="16">
+        <v>0.0</v>
+      </c>
       <c r="P8" s="16"/>
       <c r="Q8" s="16"/>
       <c r="R8" s="16"/>
@@ -2027,7 +2038,7 @@
       </c>
       <c r="AZ8" s="5">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BA8" s="5">
         <f t="shared" si="2"/>
@@ -2035,7 +2046,7 @@
       </c>
       <c r="BB8" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC8" s="5">
         <f t="shared" si="4"/>
@@ -2043,7 +2054,7 @@
       </c>
       <c r="BD8" s="5">
         <f t="shared" si="5"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="BE8" s="5">
         <f t="shared" si="6"/>
@@ -2051,7 +2062,7 @@
       </c>
       <c r="BF8" s="20">
         <f t="shared" si="7"/>
-        <v>0.5666666667</v>
+        <v>0.5454545455</v>
       </c>
       <c r="BG8" s="20"/>
     </row>
@@ -2192,7 +2203,9 @@
         <v>-2.0</v>
       </c>
       <c r="N10" s="28"/>
-      <c r="O10" s="28"/>
+      <c r="O10" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P10" s="28"/>
       <c r="Q10" s="28"/>
       <c r="R10" s="34"/>
@@ -2233,7 +2246,7 @@
       </c>
       <c r="AZ10" s="5">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BA10" s="5">
         <f t="shared" si="2"/>
@@ -2241,7 +2254,7 @@
       </c>
       <c r="BB10" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC10" s="5">
         <f t="shared" si="4"/>
@@ -2249,7 +2262,7 @@
       </c>
       <c r="BD10" s="5">
         <f t="shared" si="5"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="BE10" s="5">
         <f t="shared" si="6"/>
@@ -2257,7 +2270,7 @@
       </c>
       <c r="BF10" s="20">
         <f t="shared" si="7"/>
-        <v>0.6666666667</v>
+        <v>0.625</v>
       </c>
       <c r="BG10" s="20"/>
     </row>
@@ -2290,7 +2303,9 @@
       <c r="N11" s="28">
         <v>2.0</v>
       </c>
-      <c r="O11" s="28"/>
+      <c r="O11" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P11" s="28"/>
       <c r="Q11" s="28"/>
       <c r="R11" s="28"/>
@@ -2331,7 +2346,7 @@
       </c>
       <c r="AZ11" s="5">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BA11" s="5">
         <f t="shared" si="2"/>
@@ -2339,7 +2354,7 @@
       </c>
       <c r="BB11" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC11" s="5">
         <f t="shared" si="4"/>
@@ -2347,7 +2362,7 @@
       </c>
       <c r="BD11" s="5">
         <f t="shared" si="5"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BE11" s="5">
         <f t="shared" si="6"/>
@@ -2355,7 +2370,7 @@
       </c>
       <c r="BF11" s="20">
         <f t="shared" si="7"/>
-        <v>0.7222222222</v>
+        <v>0.6666666667</v>
       </c>
       <c r="BG11" s="20"/>
     </row>
@@ -2392,7 +2407,9 @@
       <c r="L12" s="28"/>
       <c r="M12" s="28"/>
       <c r="N12" s="28"/>
-      <c r="O12" s="28"/>
+      <c r="O12" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P12" s="28"/>
       <c r="Q12" s="28"/>
       <c r="R12" s="28"/>
@@ -2433,7 +2450,7 @@
       </c>
       <c r="AZ12" s="5">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BA12" s="5">
         <f t="shared" si="2"/>
@@ -2441,7 +2458,7 @@
       </c>
       <c r="BB12" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC12" s="5">
         <f t="shared" si="4"/>
@@ -2449,7 +2466,7 @@
       </c>
       <c r="BD12" s="5">
         <f t="shared" si="5"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="BE12" s="5">
         <f t="shared" si="6"/>
@@ -2457,7 +2474,7 @@
       </c>
       <c r="BF12" s="20">
         <f t="shared" si="7"/>
-        <v>0.5</v>
+        <v>0.4814814815</v>
       </c>
       <c r="BG12" s="20"/>
     </row>
@@ -2598,7 +2615,9 @@
       <c r="N14" s="28">
         <v>2.0</v>
       </c>
-      <c r="O14" s="28"/>
+      <c r="O14" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P14" s="28"/>
       <c r="Q14" s="28"/>
       <c r="R14" s="28"/>
@@ -2639,7 +2658,7 @@
       </c>
       <c r="AZ14" s="5">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BA14" s="5">
         <f t="shared" si="2"/>
@@ -2647,7 +2666,7 @@
       </c>
       <c r="BB14" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC14" s="5">
         <f t="shared" si="4"/>
@@ -2655,7 +2674,7 @@
       </c>
       <c r="BD14" s="5">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BE14" s="5">
         <f t="shared" si="6"/>
@@ -2704,7 +2723,9 @@
         <v>-2.0</v>
       </c>
       <c r="N15" s="28"/>
-      <c r="O15" s="28"/>
+      <c r="O15" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P15" s="28"/>
       <c r="Q15" s="28"/>
       <c r="R15" s="28"/>
@@ -2745,7 +2766,7 @@
       </c>
       <c r="AZ15" s="5">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BA15" s="5">
         <f t="shared" si="2"/>
@@ -2753,7 +2774,7 @@
       </c>
       <c r="BB15" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC15" s="5">
         <f t="shared" si="4"/>
@@ -2761,7 +2782,7 @@
       </c>
       <c r="BD15" s="5">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BE15" s="5">
         <f t="shared" si="6"/>
@@ -2769,7 +2790,7 @@
       </c>
       <c r="BF15" s="20">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.303030303</v>
       </c>
       <c r="BG15" s="20"/>
     </row>
@@ -2787,19 +2808,19 @@
       <c r="E16" s="28">
         <v>0.0</v>
       </c>
-      <c r="F16" s="28"/>
-      <c r="G16" s="29">
+      <c r="F16" s="28">
         <v>-2.0</v>
       </c>
-      <c r="H16" s="28">
+      <c r="G16" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="H16" s="29">
+        <v>1.0</v>
+      </c>
+      <c r="I16" s="28">
         <v>-1.0</v>
       </c>
-      <c r="I16" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="J16" s="28">
-        <v>-1.0</v>
-      </c>
+      <c r="J16" s="28"/>
       <c r="K16" s="28">
         <v>0.0</v>
       </c>
@@ -2812,7 +2833,9 @@
       <c r="N16" s="28">
         <v>-2.0</v>
       </c>
-      <c r="O16" s="28"/>
+      <c r="O16" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
@@ -2853,7 +2876,7 @@
       </c>
       <c r="AZ16" s="5">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="BA16" s="5">
         <f t="shared" si="2"/>
@@ -2861,7 +2884,7 @@
       </c>
       <c r="BB16" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC16" s="5">
         <f t="shared" si="4"/>
@@ -2869,15 +2892,15 @@
       </c>
       <c r="BD16" s="5">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BE16" s="5">
         <f t="shared" si="6"/>
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="BF16" s="20">
         <f t="shared" si="7"/>
-        <v>0.2727272727</v>
+        <v>0.2777777778</v>
       </c>
       <c r="BG16" s="20"/>
     </row>
@@ -2886,41 +2909,35 @@
         <v>71</v>
       </c>
       <c r="B17" s="27"/>
-      <c r="C17" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="D17" s="28">
-        <v>2.0</v>
-      </c>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
       <c r="E17" s="28">
         <v>0.0</v>
       </c>
-      <c r="F17" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="G17" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="H17" s="29">
-        <v>1.0</v>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28">
+        <v>-1.0</v>
       </c>
       <c r="I17" s="28">
         <v>-1.0</v>
       </c>
-      <c r="J17" s="28"/>
+      <c r="J17" s="29">
+        <v>-1.0</v>
+      </c>
       <c r="K17" s="28">
         <v>0.0</v>
       </c>
       <c r="L17" s="28">
-        <v>-4.0</v>
+        <v>4.0</v>
       </c>
       <c r="M17" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="N17" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="O17" s="28"/>
+        <v>2.0</v>
+      </c>
+      <c r="N17" s="28"/>
+      <c r="O17" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P17" s="28"/>
       <c r="Q17" s="28"/>
       <c r="R17" s="28"/>
@@ -2961,7 +2978,7 @@
       </c>
       <c r="AZ17" s="5">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="BA17" s="5">
         <f t="shared" si="2"/>
@@ -2973,7 +2990,7 @@
       </c>
       <c r="BC17" s="5">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BD17" s="5">
         <f t="shared" si="5"/>
@@ -2981,11 +2998,11 @@
       </c>
       <c r="BE17" s="5">
         <f t="shared" si="6"/>
-        <v>-10</v>
+        <v>3</v>
       </c>
       <c r="BF17" s="20">
         <f t="shared" si="7"/>
-        <v>0.2727272727</v>
+        <v>0.375</v>
       </c>
       <c r="BG17" s="20"/>
     </row>
@@ -2994,33 +3011,35 @@
         <v>72</v>
       </c>
       <c r="B18" s="27"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
+      <c r="C18" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="28">
+        <v>-2.0</v>
+      </c>
       <c r="E18" s="28">
         <v>0.0</v>
       </c>
       <c r="F18" s="28"/>
       <c r="G18" s="28"/>
-      <c r="H18" s="28">
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28">
         <v>-1.0</v>
       </c>
-      <c r="I18" s="28">
-        <v>-1.0</v>
-      </c>
-      <c r="J18" s="29">
-        <v>-1.0</v>
-      </c>
-      <c r="K18" s="28">
+      <c r="K18" s="28"/>
+      <c r="L18" s="29">
+        <v>4.0</v>
+      </c>
+      <c r="M18" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="N18" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="O18" s="28">
         <v>0.0</v>
       </c>
-      <c r="L18" s="28">
-        <v>4.0</v>
-      </c>
-      <c r="M18" s="28">
-        <v>2.0</v>
-      </c>
-      <c r="N18" s="28"/>
-      <c r="O18" s="28"/>
       <c r="P18" s="28"/>
       <c r="Q18" s="28"/>
       <c r="R18" s="28"/>
@@ -3061,7 +3080,7 @@
       </c>
       <c r="AZ18" s="5">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BA18" s="5">
         <f t="shared" si="2"/>
@@ -3069,7 +3088,7 @@
       </c>
       <c r="BB18" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC18" s="5">
         <f t="shared" si="4"/>
@@ -3077,15 +3096,15 @@
       </c>
       <c r="BD18" s="5">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BE18" s="5">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BF18" s="20">
         <f t="shared" si="7"/>
-        <v>0.380952381</v>
+        <v>0.375</v>
       </c>
       <c r="BG18" s="20"/>
     </row>
@@ -3098,27 +3117,35 @@
         <v>0.0</v>
       </c>
       <c r="D19" s="28">
-        <v>-2.0</v>
+        <v>2.0</v>
       </c>
       <c r="E19" s="28">
         <v>0.0</v>
       </c>
       <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
+      <c r="G19" s="29">
+        <v>-2.0</v>
+      </c>
+      <c r="H19" s="28">
+        <v>-1.0</v>
+      </c>
+      <c r="I19" s="28">
+        <v>1.0</v>
+      </c>
       <c r="J19" s="28">
         <v>-1.0</v>
       </c>
-      <c r="K19" s="28"/>
-      <c r="L19" s="29">
-        <v>4.0</v>
+      <c r="K19" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="L19" s="28">
+        <v>-4.0</v>
       </c>
       <c r="M19" s="28">
         <v>-2.0</v>
       </c>
       <c r="N19" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="O19" s="28"/>
       <c r="P19" s="28"/>
@@ -3161,7 +3188,7 @@
       </c>
       <c r="AZ19" s="5">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="BA19" s="5">
         <f t="shared" si="2"/>
@@ -3169,23 +3196,23 @@
       </c>
       <c r="BB19" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC19" s="5">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD19" s="5">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BE19" s="5">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>-9</v>
       </c>
       <c r="BF19" s="20">
         <f t="shared" si="7"/>
-        <v>0.380952381</v>
+        <v>0.2727272727</v>
       </c>
       <c r="BG19" s="20"/>
     </row>
@@ -3214,7 +3241,9 @@
       <c r="N20" s="28">
         <v>2.0</v>
       </c>
-      <c r="O20" s="28"/>
+      <c r="O20" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P20" s="28"/>
       <c r="Q20" s="28"/>
       <c r="R20" s="28"/>
@@ -3255,7 +3284,7 @@
       </c>
       <c r="AZ20" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BA20" s="5">
         <f t="shared" si="2"/>
@@ -3263,7 +3292,7 @@
       </c>
       <c r="BB20" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC20" s="5">
         <f t="shared" si="4"/>
@@ -3271,7 +3300,7 @@
       </c>
       <c r="BD20" s="5">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BE20" s="5">
         <f t="shared" si="6"/>
@@ -3279,7 +3308,7 @@
       </c>
       <c r="BF20" s="20">
         <f t="shared" si="7"/>
-        <v>0.5833333333</v>
+        <v>0.5333333333</v>
       </c>
       <c r="BG20" s="20"/>
     </row>
@@ -3290,25 +3319,33 @@
       <c r="B21" s="27"/>
       <c r="C21" s="28"/>
       <c r="D21" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="E21" s="28">
-        <v>0.0</v>
-      </c>
+        <v>2.0</v>
+      </c>
+      <c r="E21" s="28"/>
       <c r="F21" s="28"/>
       <c r="G21" s="28"/>
       <c r="H21" s="28"/>
       <c r="I21" s="28">
-        <v>1.0</v>
+        <v>-1.0</v>
       </c>
       <c r="J21" s="28">
         <v>1.0</v>
       </c>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28"/>
+      <c r="K21" s="29">
+        <v>0.0</v>
+      </c>
+      <c r="L21" s="28">
+        <v>-4.0</v>
+      </c>
+      <c r="M21" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="N21" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="O21" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P21" s="28"/>
       <c r="Q21" s="28"/>
       <c r="R21" s="28"/>
@@ -3349,7 +3386,7 @@
       </c>
       <c r="AZ21" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="BA21" s="5">
         <f t="shared" si="2"/>
@@ -3357,23 +3394,23 @@
       </c>
       <c r="BB21" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC21" s="5">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BD21" s="5">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BE21" s="5">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="BF21" s="20">
         <f t="shared" si="7"/>
-        <v>0.5833333333</v>
+        <v>0.3333333333</v>
       </c>
       <c r="BG21" s="20"/>
     </row>
@@ -3384,30 +3421,24 @@
       <c r="B22" s="27"/>
       <c r="C22" s="28"/>
       <c r="D22" s="28">
-        <v>2.0</v>
-      </c>
-      <c r="E22" s="28"/>
+        <v>-2.0</v>
+      </c>
+      <c r="E22" s="28">
+        <v>0.0</v>
+      </c>
       <c r="F22" s="28"/>
       <c r="G22" s="28"/>
       <c r="H22" s="28"/>
       <c r="I22" s="28">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="J22" s="28">
         <v>1.0</v>
       </c>
-      <c r="K22" s="29">
-        <v>0.0</v>
-      </c>
-      <c r="L22" s="28">
-        <v>-4.0</v>
-      </c>
-      <c r="M22" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="N22" s="28">
-        <v>-2.0</v>
-      </c>
+      <c r="K22" s="28"/>
+      <c r="L22" s="28"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
       <c r="O22" s="28"/>
       <c r="P22" s="28"/>
       <c r="Q22" s="28"/>
@@ -3449,7 +3480,7 @@
       </c>
       <c r="AZ22" s="5">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="BA22" s="5">
         <f t="shared" si="2"/>
@@ -3461,7 +3492,7 @@
       </c>
       <c r="BC22" s="5">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BD22" s="5">
         <f t="shared" si="5"/>
@@ -3469,11 +3500,11 @@
       </c>
       <c r="BE22" s="5">
         <f t="shared" si="6"/>
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="BF22" s="20">
         <f t="shared" si="7"/>
-        <v>0.3333333333</v>
+        <v>0.5833333333</v>
       </c>
       <c r="BG22" s="20"/>
     </row>
@@ -3592,7 +3623,9 @@
       </c>
       <c r="M24" s="28"/>
       <c r="N24" s="28"/>
-      <c r="O24" s="28"/>
+      <c r="O24" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P24" s="28"/>
       <c r="Q24" s="28"/>
       <c r="R24" s="28"/>
@@ -3633,7 +3666,7 @@
       </c>
       <c r="AZ24" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BA24" s="5">
         <f t="shared" si="2"/>
@@ -3641,7 +3674,7 @@
       </c>
       <c r="BB24" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC24" s="5">
         <f t="shared" si="4"/>
@@ -3649,7 +3682,7 @@
       </c>
       <c r="BD24" s="5">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BE24" s="5">
         <f t="shared" si="6"/>
@@ -3657,7 +3690,7 @@
       </c>
       <c r="BF24" s="20">
         <f t="shared" si="7"/>
-        <v>0.4166666667</v>
+        <v>0.4</v>
       </c>
       <c r="BG24" s="20"/>
     </row>
@@ -3682,7 +3715,9 @@
       <c r="N25" s="29">
         <v>2.0</v>
       </c>
-      <c r="O25" s="28"/>
+      <c r="O25" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P25" s="28"/>
       <c r="Q25" s="28"/>
       <c r="R25" s="28"/>
@@ -3723,7 +3758,7 @@
       </c>
       <c r="AZ25" s="5">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BA25" s="5">
         <f t="shared" si="2"/>
@@ -3731,7 +3766,7 @@
       </c>
       <c r="BB25" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC25" s="5">
         <f t="shared" si="4"/>
@@ -3739,7 +3774,7 @@
       </c>
       <c r="BD25" s="5">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BE25" s="5">
         <f t="shared" si="6"/>
@@ -3747,7 +3782,7 @@
       </c>
       <c r="BF25" s="20">
         <f t="shared" si="7"/>
-        <v>0.6666666667</v>
+        <v>0.5555555556</v>
       </c>
       <c r="BG25" s="20"/>
     </row>
@@ -4405,7 +4440,7 @@
       </c>
       <c r="BG32" s="20"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33">
       <c r="A33" s="37" t="s">
         <v>87</v>
       </c>
@@ -4981,7 +5016,7 @@
       <c r="AW39" s="28"/>
       <c r="AX39" s="28"/>
       <c r="AY39" s="19">
-        <v>30.0</v>
+        <v>35.0</v>
       </c>
       <c r="AZ39" s="5">
         <f t="shared" si="1"/>
@@ -5069,7 +5104,7 @@
       <c r="AW40" s="28"/>
       <c r="AX40" s="28"/>
       <c r="AY40" s="19">
-        <v>31.0</v>
+        <v>36.0</v>
       </c>
       <c r="AZ40" s="5">
         <f t="shared" si="1"/>
@@ -5159,7 +5194,7 @@
       </c>
       <c r="O41" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="P41" s="34">
         <f t="shared" si="8"/>
@@ -5348,7 +5383,9 @@
       <c r="N42" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="O42" s="41"/>
+      <c r="O42" s="41" t="s">
+        <v>107</v>
+      </c>
       <c r="P42" s="5"/>
       <c r="Q42" s="5"/>
       <c r="R42" s="5"/>
@@ -25748,32 +25785,32 @@
         <v>1</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F1" s="45" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G1" s="45" t="s">
         <v>56</v>
       </c>
       <c r="I1" s="45" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J1" s="45" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="37" t="s">
         <v>64</v>
       </c>
       <c r="B2" s="45">
@@ -25792,44 +25829,44 @@
         <v>2.0</v>
       </c>
       <c r="G2" s="45">
-        <f t="shared" ref="G2:G35" si="1">SUM(C2*3)+D2</f>
+        <f t="shared" ref="G2:G30" si="1">SUM(C2*3)+D2</f>
         <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B3" s="46">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C3" s="46">
         <v>1.0</v>
       </c>
       <c r="D3" s="46">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E3" s="46">
         <v>0.0</v>
       </c>
       <c r="F3" s="46">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="G3" s="46">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I3" s="45">
         <v>18.0</v>
       </c>
       <c r="J3" s="47">
         <f t="shared" ref="J3:J7" si="2">I3/B3</f>
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="s">
-        <v>114</v>
+        <v>72</v>
       </c>
       <c r="B4" s="45">
         <v>1.0</v>
@@ -25844,7 +25881,7 @@
         <v>0.0</v>
       </c>
       <c r="F4" s="45">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="G4" s="45">
         <f t="shared" si="1"/>
@@ -25860,7 +25897,7 @@
     </row>
     <row r="5">
       <c r="A5" s="26" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="B5" s="45">
         <v>1.0</v>
@@ -25953,7 +25990,7 @@
     </row>
     <row r="8">
       <c r="A8" s="32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" s="45">
         <v>1.0</v>
@@ -26079,7 +26116,7 @@
         <v>25.0</v>
       </c>
       <c r="J12" s="47">
-        <f t="shared" ref="J12:J27" si="3">I12/B12</f>
+        <f t="shared" ref="J12:J25" si="3">I12/B12</f>
         <v>25</v>
       </c>
     </row>
@@ -26117,7 +26154,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B14" s="45">
         <v>1.0</v>
@@ -26179,38 +26216,38 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B16" s="45">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C16" s="45">
         <v>0.0</v>
       </c>
       <c r="D16" s="45">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E16" s="45">
         <v>1.0</v>
       </c>
       <c r="F16" s="45">
-        <v>-1.0</v>
+        <v>-2.0</v>
       </c>
       <c r="G16" s="45">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" s="45">
         <v>23.0</v>
       </c>
       <c r="J16" s="47">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="37" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B17" s="45">
         <v>1.0</v>
@@ -26241,7 +26278,7 @@
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B18" s="45">
         <v>1.0</v>
@@ -26272,7 +26309,7 @@
     </row>
     <row r="19">
       <c r="A19" s="37" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B19" s="45">
         <v>1.0</v>
@@ -26287,7 +26324,7 @@
         <v>1.0</v>
       </c>
       <c r="F19" s="45">
-        <v>-2.0</v>
+        <v>-1.0</v>
       </c>
       <c r="G19" s="45">
         <f t="shared" si="1"/>
@@ -26303,7 +26340,7 @@
     </row>
     <row r="20">
       <c r="A20" s="37" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="45">
         <v>1.0</v>
@@ -26334,7 +26371,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="37" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B21" s="45">
         <v>1.0</v>
@@ -26458,7 +26495,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G25" s="45">
         <f t="shared" si="1"/>
@@ -26474,123 +26511,59 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="37" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="G26" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I26" s="48">
-        <v>8.0</v>
-      </c>
-      <c r="J26" s="47" t="str">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="37" t="s">
-        <v>116</v>
-      </c>
+      <c r="A27" s="37"/>
       <c r="G27" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I27" s="48">
-        <v>1.0</v>
-      </c>
-      <c r="J27" s="47" t="str">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I27" s="48"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="37" t="s">
-        <v>75</v>
+        <v>117</v>
       </c>
       <c r="G28" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I28" s="48">
-        <v>4.0</v>
+      <c r="I28" s="45">
+        <v>0.0</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G29" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I29" s="48">
-        <v>0.0</v>
-      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="37" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="G30" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I30" s="48">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="45">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I31" s="45">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="37" t="s">
-        <v>117</v>
-      </c>
-      <c r="G32" s="45">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I32" s="45">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="G33" s="45">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="G34" s="45">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="37" t="s">
-        <v>80</v>
-      </c>
-      <c r="G35" s="45">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
@@ -27918,7 +27891,7 @@
     </row>
     <row r="5">
       <c r="A5" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28">
@@ -28342,7 +28315,7 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
@@ -28545,7 +28518,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -28613,7 +28586,7 @@
     </row>
     <row r="15">
       <c r="A15" s="37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -28811,7 +28784,7 @@
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28">
@@ -29076,7 +29049,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -29644,7 +29617,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="37" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B31" s="28"/>
       <c r="C31" s="28"/>
@@ -30097,7 +30070,7 @@
       </c>
       <c r="O38" s="45">
         <f>'League Table'!O41</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="P38" s="45">
         <f>'League Table'!P41</f>
@@ -61584,7 +61557,7 @@
     </row>
     <row r="7">
       <c r="A7" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
@@ -61613,7 +61586,9 @@
       <c r="N7" s="28">
         <v>1.0</v>
       </c>
-      <c r="O7" s="28"/>
+      <c r="O7" s="28">
+        <v>1.0</v>
+      </c>
       <c r="P7" s="28"/>
       <c r="Q7" s="28"/>
       <c r="R7" s="28"/>
@@ -61652,7 +61627,7 @@
       <c r="AY7" s="28"/>
       <c r="BA7" s="45">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -61974,7 +61949,7 @@
     </row>
     <row r="13">
       <c r="A13" s="37" t="s">
-        <v>126</v>
+        <v>78</v>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -61983,17 +61958,17 @@
       <c r="F13" s="28"/>
       <c r="G13" s="28"/>
       <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
+      <c r="I13" s="28">
+        <v>1.0</v>
+      </c>
       <c r="J13" s="28"/>
-      <c r="K13" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="L13" s="28">
-        <v>1.0</v>
-      </c>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
       <c r="M13" s="28"/>
       <c r="N13" s="28"/>
-      <c r="O13" s="28"/>
+      <c r="O13" s="28">
+        <v>1.0</v>
+      </c>
       <c r="P13" s="28"/>
       <c r="Q13" s="28"/>
       <c r="R13" s="28"/>
@@ -62037,7 +62012,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -62048,9 +62023,11 @@
       <c r="H14" s="28"/>
       <c r="I14" s="28"/>
       <c r="J14" s="28"/>
-      <c r="K14" s="28"/>
+      <c r="K14" s="28">
+        <v>1.0</v>
+      </c>
       <c r="L14" s="28">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="M14" s="28"/>
       <c r="N14" s="28"/>
@@ -62098,7 +62075,7 @@
     </row>
     <row r="15">
       <c r="A15" s="37" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -62111,7 +62088,7 @@
       <c r="J15" s="28"/>
       <c r="K15" s="28"/>
       <c r="L15" s="28">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M15" s="28"/>
       <c r="N15" s="28"/>
@@ -62154,12 +62131,12 @@
       <c r="AY15" s="28"/>
       <c r="BA15" s="45">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B16" s="28"/>
       <c r="C16" s="28"/>
@@ -62168,12 +62145,12 @@
       <c r="F16" s="28"/>
       <c r="G16" s="28"/>
       <c r="H16" s="28"/>
-      <c r="I16" s="28">
-        <v>1.0</v>
-      </c>
+      <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="28"/>
-      <c r="L16" s="28"/>
+      <c r="L16" s="28">
+        <v>1.0</v>
+      </c>
       <c r="M16" s="28"/>
       <c r="N16" s="28"/>
       <c r="O16" s="28"/>
@@ -62464,7 +62441,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28">
@@ -62708,7 +62685,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -62767,7 +62744,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B26" s="28"/>
       <c r="C26" s="28"/>
@@ -62826,7 +62803,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="37" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
@@ -63584,7 +63561,7 @@
       </c>
       <c r="O39" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P39" s="5">
         <f t="shared" si="2"/>
@@ -63732,7 +63709,7 @@
       </c>
       <c r="BA39" s="45">
         <f>SUM(B39:AZ39)</f>
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1"/>
@@ -65110,17 +65087,25 @@
       <c r="A16" s="50">
         <v>14.0</v>
       </c>
-      <c r="B16" s="50"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
+      <c r="B16" s="50" t="s">
+        <v>176</v>
+      </c>
+      <c r="C16" s="50" t="s">
+        <v>177</v>
+      </c>
+      <c r="D16" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>135</v>
+      </c>
       <c r="G16" s="50"/>
       <c r="H16" s="5" t="s">
         <v>168</v>
       </c>
       <c r="I16" s="5"/>
       <c r="K16" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="5" t="s">
@@ -65144,7 +65129,7 @@
       </c>
       <c r="I17" s="5"/>
       <c r="K17" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L17" s="5"/>
       <c r="M17" s="5" t="s">
@@ -65225,12 +65210,12 @@
       <c r="D21" s="50"/>
       <c r="E21" s="50"/>
       <c r="G21" s="50"/>
-      <c r="H21" s="68"/>
+      <c r="H21" s="67"/>
       <c r="I21" s="5"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N21" s="66">
         <v>1.0</v>
@@ -65285,12 +65270,12 @@
       <c r="D24" s="50"/>
       <c r="E24" s="50"/>
       <c r="G24" s="50"/>
-      <c r="H24" s="68"/>
+      <c r="H24" s="67"/>
       <c r="I24" s="5"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="N24" s="66">
         <v>1.0</v>
@@ -65330,7 +65315,7 @@
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N26" s="66">
         <v>1.0</v>

</xml_diff>

<commit_message>
103 Week 15 update
</commit_message>
<xml_diff>
--- a/data/latest_data.xlsx
+++ b/data/latest_data.xlsx
@@ -15,14 +15,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="Q8pwG3tm1Blk2/1BcBGXSUPrEhsW2sZE0Hv4sE5tRhM="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="g32p3CLdJI2eBI3NmTEKUZOqtND4GUFAPvTklUKpY+Q="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="186">
   <si>
     <t>MARLOW DUKES 2025</t>
   </si>
@@ -228,6 +228,9 @@
     <t>SWAMPY</t>
   </si>
   <si>
+    <t>ARTIST</t>
+  </si>
+  <si>
     <t>ZIGZAG</t>
   </si>
   <si>
@@ -246,13 +249,16 @@
     <t>BRUCE</t>
   </si>
   <si>
+    <t>CARLOS</t>
+  </si>
+  <si>
     <t>DWARF</t>
   </si>
   <si>
-    <t>ARTIST</t>
+    <t>BANKSY</t>
   </si>
   <si>
-    <t>BANKSY</t>
+    <t>TONY W</t>
   </si>
   <si>
     <t>GUEST 2</t>
@@ -261,16 +267,10 @@
     <t>FLO</t>
   </si>
   <si>
-    <t>CARLOS</t>
-  </si>
-  <si>
     <t>TOY BOY</t>
   </si>
   <si>
     <t>GUEST</t>
-  </si>
-  <si>
-    <t>TONY W</t>
   </si>
   <si>
     <t>CARZOLA</t>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t xml:space="preserve"> 1-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5-0</t>
   </si>
   <si>
     <t>P</t>
@@ -561,7 +564,19 @@
     <t>Moo</t>
   </si>
   <si>
+    <t>Banksy v Tony W</t>
+  </si>
+  <si>
+    <t>Lost 0-5</t>
+  </si>
+  <si>
     <t>Swampy</t>
+  </si>
+  <si>
+    <t>Banksy</t>
+  </si>
+  <si>
+    <t>Captain Kirk</t>
   </si>
   <si>
     <t>Tony W</t>
@@ -792,7 +807,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="70">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -915,6 +930,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -927,21 +945,20 @@
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -1670,7 +1687,9 @@
       <c r="O5" s="17">
         <v>0.0</v>
       </c>
-      <c r="P5" s="16"/>
+      <c r="P5" s="16">
+        <v>5.0</v>
+      </c>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
       <c r="S5" s="16"/>
@@ -1710,11 +1729,11 @@
       </c>
       <c r="AZ5" s="5">
         <f t="shared" ref="AZ5:AZ40" si="1">COUNT(B5:AX5)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BA5" s="5">
         <f t="shared" ref="BA5:BA40" si="2">COUNTIF($B5:$AX5, "&gt;=1")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BB5" s="5">
         <f t="shared" ref="BB5:BB40" si="3">COUNTIF($B5:$AX5, "0")</f>
@@ -1726,15 +1745,15 @@
       </c>
       <c r="BD5" s="5">
         <f t="shared" ref="BD5:BD40" si="5">SUM(BA5*3)+BB5</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="BE5" s="5">
         <f t="shared" ref="BE5:BE40" si="6">SUM(B5:AX5)</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="BF5" s="20">
         <f t="shared" ref="BF5:BF40" si="7">SUM(BA5*3+BB5*1)/SUM(AZ5*3)</f>
-        <v>0.641025641</v>
+        <v>0.6666666667</v>
       </c>
       <c r="BG5" s="20"/>
     </row>
@@ -1778,7 +1797,9 @@
       <c r="O6" s="23">
         <v>0.0</v>
       </c>
-      <c r="P6" s="23"/>
+      <c r="P6" s="23">
+        <v>5.0</v>
+      </c>
       <c r="Q6" s="23"/>
       <c r="R6" s="23"/>
       <c r="S6" s="23"/>
@@ -1818,11 +1839,11 @@
       </c>
       <c r="AZ6" s="5">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="BA6" s="5">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BB6" s="5">
         <f t="shared" si="3"/>
@@ -1834,15 +1855,15 @@
       </c>
       <c r="BD6" s="5">
         <f t="shared" si="5"/>
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="BE6" s="5">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="BF6" s="20">
         <f t="shared" si="7"/>
-        <v>0.5757575758</v>
+        <v>0.6111111111</v>
       </c>
       <c r="BG6" s="20"/>
     </row>
@@ -1890,7 +1911,9 @@
       <c r="O7" s="29">
         <v>0.0</v>
       </c>
-      <c r="P7" s="28"/>
+      <c r="P7" s="28">
+        <v>5.0</v>
+      </c>
       <c r="Q7" s="28"/>
       <c r="R7" s="28"/>
       <c r="S7" s="28"/>
@@ -1930,11 +1953,11 @@
       </c>
       <c r="AZ7" s="5">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BA7" s="5">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BB7" s="5">
         <f t="shared" si="3"/>
@@ -1946,15 +1969,15 @@
       </c>
       <c r="BD7" s="5">
         <f t="shared" si="5"/>
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="BE7" s="5">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="BF7" s="20">
         <f t="shared" si="7"/>
-        <v>0.4871794872</v>
+        <v>0.5238095238</v>
       </c>
       <c r="BG7" s="20"/>
     </row>
@@ -1998,7 +2021,9 @@
       <c r="O8" s="16">
         <v>0.0</v>
       </c>
-      <c r="P8" s="16"/>
+      <c r="P8" s="16">
+        <v>5.0</v>
+      </c>
       <c r="Q8" s="16"/>
       <c r="R8" s="16"/>
       <c r="S8" s="16"/>
@@ -2038,11 +2063,11 @@
       </c>
       <c r="AZ8" s="5">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="BA8" s="5">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BB8" s="5">
         <f t="shared" si="3"/>
@@ -2054,15 +2079,15 @@
       </c>
       <c r="BD8" s="5">
         <f t="shared" si="5"/>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="BE8" s="5">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="BF8" s="20">
         <f t="shared" si="7"/>
-        <v>0.5454545455</v>
+        <v>0.5833333333</v>
       </c>
       <c r="BG8" s="20"/>
     </row>
@@ -2410,7 +2435,9 @@
       <c r="O12" s="28">
         <v>0.0</v>
       </c>
-      <c r="P12" s="28"/>
+      <c r="P12" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q12" s="28"/>
       <c r="R12" s="28"/>
       <c r="S12" s="28"/>
@@ -2450,7 +2477,7 @@
       </c>
       <c r="AZ12" s="5">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BA12" s="5">
         <f t="shared" si="2"/>
@@ -2462,7 +2489,7 @@
       </c>
       <c r="BC12" s="5">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BD12" s="5">
         <f t="shared" si="5"/>
@@ -2470,11 +2497,11 @@
       </c>
       <c r="BE12" s="5">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="BF12" s="20">
         <f t="shared" si="7"/>
-        <v>0.4814814815</v>
+        <v>0.4333333333</v>
       </c>
       <c r="BG12" s="20"/>
     </row>
@@ -2585,40 +2612,38 @@
         <v>68</v>
       </c>
       <c r="B14" s="27"/>
-      <c r="C14" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="28"/>
-      <c r="E14" s="29">
-        <v>0.0</v>
-      </c>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="E14" s="28"/>
       <c r="F14" s="28"/>
-      <c r="G14" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="H14" s="28">
-        <v>-1.0</v>
-      </c>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="28">
         <v>-1.0</v>
       </c>
       <c r="J14" s="28">
-        <v>-1.0</v>
-      </c>
-      <c r="K14" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="K14" s="29">
         <v>0.0</v>
       </c>
-      <c r="L14" s="28"/>
+      <c r="L14" s="28">
+        <v>-4.0</v>
+      </c>
       <c r="M14" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="N14" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="O14" s="28">
         <v>0.0</v>
       </c>
-      <c r="P14" s="28"/>
+      <c r="P14" s="28">
+        <v>5.0</v>
+      </c>
       <c r="Q14" s="28"/>
       <c r="R14" s="28"/>
       <c r="S14" s="28"/>
@@ -2658,15 +2683,15 @@
       </c>
       <c r="AZ14" s="5">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="BA14" s="5">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB14" s="5">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BC14" s="5">
         <f t="shared" si="4"/>
@@ -2674,7 +2699,7 @@
       </c>
       <c r="BD14" s="5">
         <f t="shared" si="5"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BE14" s="5">
         <f t="shared" si="6"/>
@@ -2682,7 +2707,7 @@
       </c>
       <c r="BF14" s="20">
         <f t="shared" si="7"/>
-        <v>0.3333333333</v>
+        <v>0.4074074074</v>
       </c>
       <c r="BG14" s="20"/>
     </row>
@@ -2694,39 +2719,39 @@
       <c r="C15" s="28">
         <v>0.0</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="28"/>
+      <c r="E15" s="29">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28">
         <v>-2.0</v>
       </c>
-      <c r="E15" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="F15" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="G15" s="28">
-        <v>2.0</v>
-      </c>
       <c r="H15" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="I15" s="29">
         <v>-1.0</v>
       </c>
-      <c r="J15" s="28"/>
+      <c r="I15" s="28">
+        <v>-1.0</v>
+      </c>
+      <c r="J15" s="28">
+        <v>-1.0</v>
+      </c>
       <c r="K15" s="28">
         <v>0.0</v>
       </c>
-      <c r="L15" s="28">
-        <v>-4.0</v>
-      </c>
+      <c r="L15" s="28"/>
       <c r="M15" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="N15" s="28"/>
+        <v>2.0</v>
+      </c>
+      <c r="N15" s="28">
+        <v>2.0</v>
+      </c>
       <c r="O15" s="28">
         <v>0.0</v>
       </c>
-      <c r="P15" s="28"/>
+      <c r="P15" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q15" s="28"/>
       <c r="R15" s="28"/>
       <c r="S15" s="28"/>
@@ -2786,7 +2811,7 @@
       </c>
       <c r="BE15" s="5">
         <f t="shared" si="6"/>
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="BF15" s="20">
         <f t="shared" si="7"/>
@@ -2803,7 +2828,7 @@
         <v>0.0</v>
       </c>
       <c r="D16" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="E16" s="28">
         <v>0.0</v>
@@ -2812,12 +2837,12 @@
         <v>-2.0</v>
       </c>
       <c r="G16" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="H16" s="29">
+        <v>2.0</v>
+      </c>
+      <c r="H16" s="28">
         <v>1.0</v>
       </c>
-      <c r="I16" s="28">
+      <c r="I16" s="29">
         <v>-1.0</v>
       </c>
       <c r="J16" s="28"/>
@@ -2830,9 +2855,7 @@
       <c r="M16" s="28">
         <v>-2.0</v>
       </c>
-      <c r="N16" s="28">
-        <v>-2.0</v>
-      </c>
+      <c r="N16" s="28"/>
       <c r="O16" s="28">
         <v>0.0</v>
       </c>
@@ -2876,7 +2899,7 @@
       </c>
       <c r="AZ16" s="5">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BA16" s="5">
         <f t="shared" si="2"/>
@@ -2888,7 +2911,7 @@
       </c>
       <c r="BC16" s="5">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BD16" s="5">
         <f t="shared" si="5"/>
@@ -2896,11 +2919,11 @@
       </c>
       <c r="BE16" s="5">
         <f t="shared" si="6"/>
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="BF16" s="20">
         <f t="shared" si="7"/>
-        <v>0.2777777778</v>
+        <v>0.303030303</v>
       </c>
       <c r="BG16" s="20"/>
     </row>
@@ -2909,32 +2932,40 @@
         <v>71</v>
       </c>
       <c r="B17" s="27"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
+      <c r="C17" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="28">
+        <v>2.0</v>
+      </c>
       <c r="E17" s="28">
         <v>0.0</v>
       </c>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28">
-        <v>-1.0</v>
+      <c r="F17" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="G17" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="H17" s="29">
+        <v>1.0</v>
       </c>
       <c r="I17" s="28">
         <v>-1.0</v>
       </c>
-      <c r="J17" s="29">
-        <v>-1.0</v>
-      </c>
+      <c r="J17" s="28"/>
       <c r="K17" s="28">
         <v>0.0</v>
       </c>
       <c r="L17" s="28">
-        <v>4.0</v>
+        <v>-4.0</v>
       </c>
       <c r="M17" s="28">
-        <v>2.0</v>
-      </c>
-      <c r="N17" s="28"/>
+        <v>-2.0</v>
+      </c>
+      <c r="N17" s="28">
+        <v>-2.0</v>
+      </c>
       <c r="O17" s="28">
         <v>0.0</v>
       </c>
@@ -2978,7 +3009,7 @@
       </c>
       <c r="AZ17" s="5">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="BA17" s="5">
         <f t="shared" si="2"/>
@@ -2986,23 +3017,23 @@
       </c>
       <c r="BB17" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC17" s="5">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD17" s="5">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BE17" s="5">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>-10</v>
       </c>
       <c r="BF17" s="20">
         <f t="shared" si="7"/>
-        <v>0.375</v>
+        <v>0.2777777778</v>
       </c>
       <c r="BG17" s="20"/>
     </row>
@@ -3011,32 +3042,32 @@
         <v>72</v>
       </c>
       <c r="B18" s="27"/>
-      <c r="C18" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="D18" s="28">
-        <v>-2.0</v>
-      </c>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
       <c r="E18" s="28">
         <v>0.0</v>
       </c>
       <c r="F18" s="28"/>
       <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28">
+      <c r="H18" s="28">
         <v>-1.0</v>
       </c>
-      <c r="K18" s="28"/>
-      <c r="L18" s="29">
+      <c r="I18" s="28">
+        <v>-1.0</v>
+      </c>
+      <c r="J18" s="29">
+        <v>-1.0</v>
+      </c>
+      <c r="K18" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="L18" s="28">
         <v>4.0</v>
       </c>
       <c r="M18" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="N18" s="28">
         <v>2.0</v>
       </c>
+      <c r="N18" s="28"/>
       <c r="O18" s="28">
         <v>0.0</v>
       </c>
@@ -3100,7 +3131,7 @@
       </c>
       <c r="BE18" s="5">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF18" s="20">
         <f t="shared" si="7"/>
@@ -3117,38 +3148,34 @@
         <v>0.0</v>
       </c>
       <c r="D19" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="E19" s="28">
         <v>0.0</v>
       </c>
       <c r="F19" s="28"/>
-      <c r="G19" s="29">
-        <v>-2.0</v>
-      </c>
-      <c r="H19" s="28">
-        <v>-1.0</v>
-      </c>
-      <c r="I19" s="28">
-        <v>1.0</v>
-      </c>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
       <c r="J19" s="28">
         <v>-1.0</v>
       </c>
-      <c r="K19" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="L19" s="28">
-        <v>-4.0</v>
+      <c r="K19" s="28"/>
+      <c r="L19" s="29">
+        <v>4.0</v>
       </c>
       <c r="M19" s="28">
         <v>-2.0</v>
       </c>
       <c r="N19" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="O19" s="28"/>
-      <c r="P19" s="28"/>
+        <v>2.0</v>
+      </c>
+      <c r="O19" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="P19" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q19" s="28"/>
       <c r="R19" s="28"/>
       <c r="S19" s="28"/>
@@ -3188,7 +3215,7 @@
       </c>
       <c r="AZ19" s="5">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="BA19" s="5">
         <f t="shared" si="2"/>
@@ -3200,7 +3227,7 @@
       </c>
       <c r="BC19" s="5">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BD19" s="5">
         <f t="shared" si="5"/>
@@ -3208,11 +3235,11 @@
       </c>
       <c r="BE19" s="5">
         <f t="shared" si="6"/>
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="BF19" s="20">
         <f t="shared" si="7"/>
-        <v>0.2727272727</v>
+        <v>0.3333333333</v>
       </c>
       <c r="BG19" s="20"/>
     </row>
@@ -3221,30 +3248,44 @@
         <v>74</v>
       </c>
       <c r="B20" s="27"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
+      <c r="C20" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="E20" s="28">
+        <v>0.0</v>
+      </c>
       <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
+      <c r="G20" s="29">
+        <v>-2.0</v>
+      </c>
+      <c r="H20" s="28">
+        <v>-1.0</v>
+      </c>
+      <c r="I20" s="28">
+        <v>1.0</v>
+      </c>
       <c r="J20" s="28">
         <v>-1.0</v>
       </c>
-      <c r="K20" s="29">
+      <c r="K20" s="28">
         <v>0.0</v>
       </c>
-      <c r="L20" s="28"/>
+      <c r="L20" s="28">
+        <v>-4.0</v>
+      </c>
       <c r="M20" s="28">
-        <v>2.0</v>
+        <v>-2.0</v>
       </c>
       <c r="N20" s="28">
-        <v>2.0</v>
-      </c>
-      <c r="O20" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="P20" s="28"/>
+        <v>-2.0</v>
+      </c>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q20" s="28"/>
       <c r="R20" s="28"/>
       <c r="S20" s="28"/>
@@ -3284,7 +3325,7 @@
       </c>
       <c r="AZ20" s="5">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="BA20" s="5">
         <f t="shared" si="2"/>
@@ -3292,23 +3333,23 @@
       </c>
       <c r="BB20" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC20" s="5">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="BD20" s="5">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BE20" s="5">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>-14</v>
       </c>
       <c r="BF20" s="20">
         <f t="shared" si="7"/>
-        <v>0.5333333333</v>
+        <v>0.25</v>
       </c>
       <c r="BG20" s="20"/>
     </row>
@@ -3317,36 +3358,28 @@
         <v>75</v>
       </c>
       <c r="B21" s="27"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28">
-        <v>2.0</v>
-      </c>
+      <c r="C21" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="28"/>
       <c r="E21" s="28"/>
       <c r="F21" s="28"/>
       <c r="G21" s="28"/>
       <c r="H21" s="28"/>
-      <c r="I21" s="28">
-        <v>-1.0</v>
-      </c>
-      <c r="J21" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="K21" s="29">
-        <v>0.0</v>
-      </c>
-      <c r="L21" s="28">
-        <v>-4.0</v>
-      </c>
-      <c r="M21" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="N21" s="28">
-        <v>-2.0</v>
+      <c r="I21" s="28"/>
+      <c r="J21" s="28"/>
+      <c r="K21" s="28"/>
+      <c r="L21" s="28"/>
+      <c r="M21" s="28"/>
+      <c r="N21" s="29">
+        <v>2.0</v>
       </c>
       <c r="O21" s="28">
         <v>0.0</v>
       </c>
-      <c r="P21" s="28"/>
+      <c r="P21" s="28">
+        <v>5.0</v>
+      </c>
       <c r="Q21" s="28"/>
       <c r="R21" s="28"/>
       <c r="S21" s="28"/>
@@ -3386,7 +3419,7 @@
       </c>
       <c r="AZ21" s="5">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="BA21" s="5">
         <f t="shared" si="2"/>
@@ -3398,7 +3431,7 @@
       </c>
       <c r="BC21" s="5">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BD21" s="5">
         <f t="shared" si="5"/>
@@ -3406,11 +3439,11 @@
       </c>
       <c r="BE21" s="5">
         <f t="shared" si="6"/>
-        <v>-6</v>
+        <v>7</v>
       </c>
       <c r="BF21" s="20">
         <f t="shared" si="7"/>
-        <v>0.3333333333</v>
+        <v>0.6666666667</v>
       </c>
       <c r="BG21" s="20"/>
     </row>
@@ -3420,26 +3453,28 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="28"/>
-      <c r="D22" s="28">
-        <v>-2.0</v>
-      </c>
-      <c r="E22" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
       <c r="F22" s="28"/>
       <c r="G22" s="28"/>
       <c r="H22" s="28"/>
-      <c r="I22" s="28">
-        <v>1.0</v>
-      </c>
+      <c r="I22" s="28"/>
       <c r="J22" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="K22" s="28"/>
+        <v>-1.0</v>
+      </c>
+      <c r="K22" s="29">
+        <v>0.0</v>
+      </c>
       <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28"/>
+      <c r="M22" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="N22" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="O22" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P22" s="28"/>
       <c r="Q22" s="28"/>
       <c r="R22" s="28"/>
@@ -3480,7 +3515,7 @@
       </c>
       <c r="AZ22" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BA22" s="5">
         <f t="shared" si="2"/>
@@ -3488,7 +3523,7 @@
       </c>
       <c r="BB22" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC22" s="5">
         <f t="shared" si="4"/>
@@ -3496,15 +3531,15 @@
       </c>
       <c r="BD22" s="5">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BE22" s="5">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BF22" s="20">
         <f t="shared" si="7"/>
-        <v>0.5833333333</v>
+        <v>0.5333333333</v>
       </c>
       <c r="BG22" s="20"/>
     </row>
@@ -3514,23 +3549,29 @@
       </c>
       <c r="B23" s="27"/>
       <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
+      <c r="D23" s="28">
+        <v>-2.0</v>
+      </c>
+      <c r="E23" s="28">
+        <v>0.0</v>
+      </c>
       <c r="F23" s="28"/>
       <c r="G23" s="28"/>
       <c r="H23" s="28"/>
       <c r="I23" s="28">
         <v>1.0</v>
       </c>
-      <c r="J23" s="28"/>
+      <c r="J23" s="28">
+        <v>1.0</v>
+      </c>
       <c r="K23" s="28"/>
       <c r="L23" s="28"/>
       <c r="M23" s="28"/>
-      <c r="N23" s="28">
-        <v>2.0</v>
-      </c>
+      <c r="N23" s="28"/>
       <c r="O23" s="28"/>
-      <c r="P23" s="28"/>
+      <c r="P23" s="29">
+        <v>-5.0</v>
+      </c>
       <c r="Q23" s="28"/>
       <c r="R23" s="28"/>
       <c r="S23" s="28"/>
@@ -3570,7 +3611,7 @@
       </c>
       <c r="AZ23" s="5">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BA23" s="5">
         <f t="shared" si="2"/>
@@ -3578,23 +3619,23 @@
       </c>
       <c r="BB23" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC23" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BD23" s="5">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BE23" s="5">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>-5</v>
       </c>
       <c r="BF23" s="20">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>0.4666666667</v>
       </c>
       <c r="BG23" s="20"/>
     </row>
@@ -3603,30 +3644,26 @@
         <v>78</v>
       </c>
       <c r="B24" s="27"/>
-      <c r="C24" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="C24" s="28"/>
       <c r="D24" s="28"/>
-      <c r="E24" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="E24" s="28"/>
       <c r="F24" s="28"/>
       <c r="G24" s="28"/>
       <c r="H24" s="28"/>
-      <c r="I24" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="J24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28">
+        <v>-1.0</v>
+      </c>
       <c r="K24" s="28"/>
-      <c r="L24" s="29">
-        <v>-4.0</v>
-      </c>
-      <c r="M24" s="28"/>
+      <c r="L24" s="28"/>
+      <c r="M24" s="28">
+        <v>2.0</v>
+      </c>
       <c r="N24" s="28"/>
-      <c r="O24" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="P24" s="28"/>
+      <c r="O24" s="28"/>
+      <c r="P24" s="29">
+        <v>5.0</v>
+      </c>
       <c r="Q24" s="28"/>
       <c r="R24" s="28"/>
       <c r="S24" s="28"/>
@@ -3666,15 +3703,15 @@
       </c>
       <c r="AZ24" s="5">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BA24" s="5">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB24" s="5">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BC24" s="5">
         <f t="shared" si="4"/>
@@ -3686,11 +3723,11 @@
       </c>
       <c r="BE24" s="5">
         <f t="shared" si="6"/>
-        <v>-3</v>
+        <v>6</v>
       </c>
       <c r="BF24" s="20">
         <f t="shared" si="7"/>
-        <v>0.4</v>
+        <v>0.6666666667</v>
       </c>
       <c r="BG24" s="20"/>
     </row>
@@ -3699,25 +3736,23 @@
         <v>79</v>
       </c>
       <c r="B25" s="27"/>
-      <c r="C25" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="C25" s="28"/>
       <c r="D25" s="28"/>
       <c r="E25" s="28"/>
       <c r="F25" s="28"/>
       <c r="G25" s="28"/>
       <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
+      <c r="I25" s="28">
+        <v>1.0</v>
+      </c>
       <c r="J25" s="28"/>
       <c r="K25" s="28"/>
       <c r="L25" s="28"/>
       <c r="M25" s="28"/>
-      <c r="N25" s="29">
+      <c r="N25" s="28">
         <v>2.0</v>
       </c>
-      <c r="O25" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="O25" s="28"/>
       <c r="P25" s="28"/>
       <c r="Q25" s="28"/>
       <c r="R25" s="28"/>
@@ -3758,15 +3793,15 @@
       </c>
       <c r="AZ25" s="5">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BA25" s="5">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB25" s="5">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BC25" s="5">
         <f t="shared" si="4"/>
@@ -3774,15 +3809,15 @@
       </c>
       <c r="BD25" s="5">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BE25" s="5">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF25" s="20">
         <f t="shared" si="7"/>
-        <v>0.5555555556</v>
+        <v>1</v>
       </c>
       <c r="BG25" s="20"/>
     </row>
@@ -3791,23 +3826,29 @@
         <v>80</v>
       </c>
       <c r="B26" s="27"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28">
-        <v>2.0</v>
-      </c>
+      <c r="C26" s="28">
+        <v>0.0</v>
+      </c>
+      <c r="D26" s="28"/>
       <c r="E26" s="28">
         <v>0.0</v>
       </c>
       <c r="F26" s="28"/>
       <c r="G26" s="28"/>
       <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
+      <c r="I26" s="28">
+        <v>1.0</v>
+      </c>
       <c r="J26" s="28"/>
       <c r="K26" s="28"/>
-      <c r="L26" s="28"/>
+      <c r="L26" s="29">
+        <v>-4.0</v>
+      </c>
       <c r="M26" s="28"/>
       <c r="N26" s="28"/>
-      <c r="O26" s="28"/>
+      <c r="O26" s="28">
+        <v>0.0</v>
+      </c>
       <c r="P26" s="28"/>
       <c r="Q26" s="28"/>
       <c r="R26" s="28"/>
@@ -3848,7 +3889,7 @@
       </c>
       <c r="AZ26" s="5">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BA26" s="5">
         <f t="shared" si="2"/>
@@ -3856,23 +3897,23 @@
       </c>
       <c r="BB26" s="5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BC26" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD26" s="5">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BE26" s="5">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="BF26" s="20">
         <f t="shared" si="7"/>
-        <v>0.6666666667</v>
+        <v>0.4</v>
       </c>
       <c r="BG26" s="20"/>
     </row>
@@ -3882,25 +3923,21 @@
       </c>
       <c r="B27" s="27"/>
       <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
+      <c r="D27" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="E27" s="28">
+        <v>0.0</v>
+      </c>
       <c r="F27" s="28"/>
       <c r="G27" s="28"/>
       <c r="H27" s="28"/>
-      <c r="I27" s="28">
-        <v>-1.0</v>
-      </c>
+      <c r="I27" s="28"/>
       <c r="J27" s="28"/>
-      <c r="K27" s="28">
-        <v>0.0</v>
-      </c>
+      <c r="K27" s="28"/>
       <c r="L27" s="28"/>
-      <c r="M27" s="28">
-        <v>2.0</v>
-      </c>
-      <c r="N27" s="28">
-        <v>-2.0</v>
-      </c>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
       <c r="O27" s="28"/>
       <c r="P27" s="28"/>
       <c r="Q27" s="28"/>
@@ -3942,7 +3979,7 @@
       </c>
       <c r="AZ27" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BA27" s="5">
         <f t="shared" si="2"/>
@@ -3954,7 +3991,7 @@
       </c>
       <c r="BC27" s="5">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BD27" s="5">
         <f t="shared" si="5"/>
@@ -3962,11 +3999,11 @@
       </c>
       <c r="BE27" s="5">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="BF27" s="20">
         <f t="shared" si="7"/>
-        <v>0.3333333333</v>
+        <v>0.6666666667</v>
       </c>
       <c r="BG27" s="20"/>
     </row>
@@ -3981,16 +4018,20 @@
       <c r="F28" s="28"/>
       <c r="G28" s="28"/>
       <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28">
+      <c r="I28" s="28">
         <v>-1.0</v>
       </c>
-      <c r="K28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28">
+        <v>0.0</v>
+      </c>
       <c r="L28" s="28"/>
       <c r="M28" s="28">
         <v>2.0</v>
       </c>
-      <c r="N28" s="28"/>
+      <c r="N28" s="28">
+        <v>-2.0</v>
+      </c>
       <c r="O28" s="28"/>
       <c r="P28" s="28"/>
       <c r="Q28" s="28"/>
@@ -4032,7 +4073,7 @@
       </c>
       <c r="AZ28" s="5">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BA28" s="5">
         <f t="shared" si="2"/>
@@ -4040,23 +4081,23 @@
       </c>
       <c r="BB28" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC28" s="5">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD28" s="5">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BE28" s="5">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="BF28" s="20">
         <f t="shared" si="7"/>
-        <v>0.5</v>
+        <v>0.3333333333</v>
       </c>
       <c r="BG28" s="20"/>
     </row>
@@ -4178,7 +4219,9 @@
       <c r="M30" s="28"/>
       <c r="N30" s="28"/>
       <c r="O30" s="28"/>
-      <c r="P30" s="28"/>
+      <c r="P30" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q30" s="28"/>
       <c r="R30" s="28"/>
       <c r="S30" s="28"/>
@@ -4218,7 +4261,7 @@
       </c>
       <c r="AZ30" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BA30" s="5">
         <f t="shared" si="2"/>
@@ -4230,7 +4273,7 @@
       </c>
       <c r="BC30" s="5">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD30" s="5">
         <f t="shared" si="5"/>
@@ -4238,11 +4281,11 @@
       </c>
       <c r="BE30" s="5">
         <f t="shared" si="6"/>
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="BF30" s="20">
         <f t="shared" si="7"/>
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="BG30" s="20"/>
     </row>
@@ -4372,7 +4415,9 @@
       <c r="M32" s="28"/>
       <c r="N32" s="28"/>
       <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>-5.0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -4412,7 +4457,7 @@
       </c>
       <c r="AZ32" s="5">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BA32" s="5">
         <f t="shared" si="2"/>
@@ -4424,7 +4469,7 @@
       </c>
       <c r="BC32" s="5">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BD32" s="5">
         <f t="shared" si="5"/>
@@ -4432,15 +4477,15 @@
       </c>
       <c r="BE32" s="5">
         <f t="shared" si="6"/>
-        <v>-9</v>
+        <v>-14</v>
       </c>
       <c r="BF32" s="20">
         <f t="shared" si="7"/>
-        <v>0.09523809524</v>
+        <v>0.08333333333</v>
       </c>
       <c r="BG32" s="20"/>
     </row>
-    <row r="33">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="37" t="s">
         <v>87</v>
       </c>
@@ -5198,7 +5243,7 @@
       </c>
       <c r="P41" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q41" s="34">
         <f t="shared" si="8"/>
@@ -5386,7 +5431,9 @@
       <c r="O42" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="P42" s="5"/>
+      <c r="P42" s="5" t="s">
+        <v>108</v>
+      </c>
       <c r="Q42" s="5"/>
       <c r="R42" s="5"/>
       <c r="S42" s="41"/>
@@ -25785,28 +25832,28 @@
         <v>1</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F1" s="45" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G1" s="45" t="s">
         <v>56</v>
       </c>
       <c r="I1" s="45" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J1" s="45" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
@@ -25866,7 +25913,7 @@
     </row>
     <row r="4">
       <c r="A4" s="21" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B4" s="45">
         <v>1.0</v>
@@ -25881,7 +25928,7 @@
         <v>0.0</v>
       </c>
       <c r="F4" s="45">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="G4" s="45">
         <f t="shared" si="1"/>
@@ -25897,7 +25944,7 @@
     </row>
     <row r="5">
       <c r="A5" s="26" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="B5" s="45">
         <v>1.0</v>
@@ -25912,7 +25959,7 @@
         <v>0.0</v>
       </c>
       <c r="F5" s="45">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="G5" s="45">
         <f t="shared" si="1"/>
@@ -25928,7 +25975,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="B6" s="46">
         <v>1.0</v>
@@ -25959,7 +26006,7 @@
     </row>
     <row r="7">
       <c r="A7" s="32" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B7" s="45">
         <v>1.0</v>
@@ -25990,7 +26037,7 @@
     </row>
     <row r="8">
       <c r="A8" s="32" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B8" s="45">
         <v>1.0</v>
@@ -26005,7 +26052,7 @@
         <v>0.0</v>
       </c>
       <c r="F8" s="45">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="G8" s="45">
         <f t="shared" si="1"/>
@@ -26015,7 +26062,7 @@
     </row>
     <row r="9">
       <c r="A9" s="37" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B9" s="45">
         <v>1.0</v>
@@ -26040,7 +26087,7 @@
     </row>
     <row r="10">
       <c r="A10" s="37" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B10" s="45">
         <v>1.0</v>
@@ -26066,32 +26113,32 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="B11" s="45">
         <v>1.0</v>
       </c>
       <c r="C11" s="45">
+        <v>1.0</v>
+      </c>
+      <c r="D11" s="45">
         <v>0.0</v>
-      </c>
-      <c r="D11" s="45">
-        <v>1.0</v>
       </c>
       <c r="E11" s="45">
         <v>0.0</v>
       </c>
       <c r="F11" s="45">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G11" s="45">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11" s="47"/>
     </row>
     <row r="12">
       <c r="A12" s="37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B12" s="45">
         <v>1.0</v>
@@ -26122,7 +26169,7 @@
     </row>
     <row r="13">
       <c r="A13" s="37" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="B13" s="45">
         <v>1.0</v>
@@ -26154,7 +26201,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B14" s="45">
         <v>1.0</v>
@@ -26185,7 +26232,7 @@
     </row>
     <row r="15">
       <c r="A15" s="37" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B15" s="45">
         <v>1.0</v>
@@ -26216,10 +26263,10 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="B16" s="45">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="C16" s="45">
         <v>0.0</v>
@@ -26228,10 +26275,10 @@
         <v>1.0</v>
       </c>
       <c r="E16" s="45">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F16" s="45">
-        <v>-2.0</v>
+        <v>0.0</v>
       </c>
       <c r="G16" s="45">
         <f t="shared" si="1"/>
@@ -26242,43 +26289,43 @@
       </c>
       <c r="J16" s="47">
         <f t="shared" si="3"/>
-        <v>11.5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="37" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B17" s="45">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C17" s="45">
         <v>0.0</v>
       </c>
       <c r="D17" s="45">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E17" s="45">
         <v>1.0</v>
       </c>
       <c r="F17" s="45">
-        <v>-1.0</v>
+        <v>-2.0</v>
       </c>
       <c r="G17" s="45">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="48">
         <v>19.0</v>
       </c>
       <c r="J17" s="47">
         <f t="shared" si="3"/>
-        <v>19</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B18" s="45">
         <v>1.0</v>
@@ -26309,7 +26356,7 @@
     </row>
     <row r="19">
       <c r="A19" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" s="45">
         <v>1.0</v>
@@ -26340,7 +26387,7 @@
     </row>
     <row r="20">
       <c r="A20" s="37" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="B20" s="45">
         <v>1.0</v>
@@ -26355,7 +26402,7 @@
         <v>1.0</v>
       </c>
       <c r="F20" s="45">
-        <v>-2.0</v>
+        <v>-1.0</v>
       </c>
       <c r="G20" s="45">
         <f t="shared" si="1"/>
@@ -26371,7 +26418,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="37" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B21" s="45">
         <v>1.0</v>
@@ -26402,7 +26449,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="37" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="B22" s="45">
         <v>1.0</v>
@@ -26433,7 +26480,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="37" t="s">
-        <v>67</v>
+        <v>94</v>
       </c>
       <c r="B23" s="45">
         <v>1.0</v>
@@ -26464,7 +26511,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="37" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B24" s="45">
         <v>1.0</v>
@@ -26479,7 +26526,7 @@
         <v>1.0</v>
       </c>
       <c r="F24" s="45">
-        <v>-4.0</v>
+        <v>-2.0</v>
       </c>
       <c r="G24" s="45">
         <f t="shared" si="1"/>
@@ -26495,7 +26542,22 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="37" t="s">
-        <v>116</v>
+        <v>80</v>
+      </c>
+      <c r="B25" s="45">
+        <v>1.0</v>
+      </c>
+      <c r="C25" s="45">
+        <v>0.0</v>
+      </c>
+      <c r="D25" s="45">
+        <v>0.0</v>
+      </c>
+      <c r="E25" s="45">
+        <v>1.0</v>
+      </c>
+      <c r="F25" s="45">
+        <v>-4.0</v>
       </c>
       <c r="G25" s="45">
         <f t="shared" si="1"/>
@@ -26504,14 +26566,29 @@
       <c r="I25" s="48">
         <v>25.0</v>
       </c>
-      <c r="J25" s="47" t="str">
+      <c r="J25" s="47">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="37" t="s">
-        <v>76</v>
+        <v>77</v>
+      </c>
+      <c r="B26" s="45">
+        <v>1.0</v>
+      </c>
+      <c r="C26" s="45">
+        <v>0.0</v>
+      </c>
+      <c r="D26" s="45">
+        <v>0.0</v>
+      </c>
+      <c r="E26" s="45">
+        <v>1.0</v>
+      </c>
+      <c r="F26" s="45">
+        <v>-5.0</v>
       </c>
       <c r="G26" s="45">
         <f t="shared" si="1"/>
@@ -26522,7 +26599,9 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="37"/>
+      <c r="A27" s="37" t="s">
+        <v>117</v>
+      </c>
       <c r="G27" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -26531,7 +26610,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G28" s="45">
         <f t="shared" si="1"/>
@@ -26552,7 +26631,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G30" s="45">
         <f t="shared" si="1"/>
@@ -27704,17 +27783,17 @@
         <v>50</v>
       </c>
       <c r="AY1" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AZ1" s="6"/>
       <c r="BA1" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BB1" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="BC1" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2">
@@ -27891,7 +27970,7 @@
     </row>
     <row r="5">
       <c r="A5" s="26" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28">
@@ -28035,7 +28114,7 @@
     </row>
     <row r="7">
       <c r="A7" s="32" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
@@ -28175,7 +28254,7 @@
     </row>
     <row r="9">
       <c r="A9" s="37" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -28315,7 +28394,7 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
@@ -28383,7 +28462,7 @@
     </row>
     <row r="12">
       <c r="A12" s="37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B12" s="28"/>
       <c r="C12" s="28"/>
@@ -28518,7 +28597,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -28586,7 +28665,7 @@
     </row>
     <row r="15">
       <c r="A15" s="37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -28784,7 +28863,7 @@
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28">
@@ -28851,7 +28930,7 @@
     </row>
     <row r="19">
       <c r="A19" s="37" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="28">
@@ -29049,7 +29128,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="37" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -29179,7 +29258,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B24" s="28"/>
       <c r="C24" s="28"/>
@@ -29243,7 +29322,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="37" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -29369,7 +29448,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
@@ -29493,7 +29572,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="37" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
@@ -29617,7 +29696,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B31" s="28"/>
       <c r="C31" s="28"/>
@@ -30074,7 +30153,7 @@
       </c>
       <c r="P38" s="45">
         <f>'League Table'!P41</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q38" s="45">
         <f>'League Table'!Q41</f>
@@ -30246,7 +30325,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="45" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B40" s="45">
         <f t="shared" ref="B40:AV40" si="2">SUM(B3:B36)</f>
@@ -61188,7 +61267,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1"/>
       <c r="D1" s="2"/>
@@ -61353,10 +61432,10 @@
         <v>50</v>
       </c>
       <c r="AY3" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BA3" s="55" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
@@ -61445,7 +61524,9 @@
         <v>3.0</v>
       </c>
       <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
+      <c r="P5" s="56">
+        <v>1.0</v>
+      </c>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
       <c r="S5" s="16"/>
@@ -61483,29 +61564,29 @@
       <c r="AY5" s="16"/>
       <c r="BA5" s="45">
         <f t="shared" ref="BA5:BA37" si="1">SUM(B5:AY5)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="57" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57">
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58">
         <v>1.0</v>
       </c>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57">
+      <c r="H6" s="58"/>
+      <c r="I6" s="58">
         <v>1.0</v>
       </c>
-      <c r="J6" s="57">
+      <c r="J6" s="58">
         <v>3.0</v>
       </c>
-      <c r="K6" s="58"/>
+      <c r="K6" s="59"/>
       <c r="L6" s="34">
         <v>4.0</v>
       </c>
@@ -61557,7 +61638,7 @@
     </row>
     <row r="7">
       <c r="A7" s="26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
@@ -61574,7 +61655,7 @@
       </c>
       <c r="I7" s="28"/>
       <c r="J7" s="28"/>
-      <c r="K7" s="59">
+      <c r="K7" s="60">
         <v>1.0</v>
       </c>
       <c r="L7" s="28">
@@ -61632,90 +61713,94 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="K8" s="60"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16">
+        <v>78</v>
+      </c>
+      <c r="B8" s="61"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="63">
         <v>1.0</v>
       </c>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="16"/>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="16"/>
-      <c r="AD8" s="16"/>
-      <c r="AE8" s="16"/>
-      <c r="AF8" s="16"/>
-      <c r="AG8" s="16"/>
-      <c r="AH8" s="16"/>
-      <c r="AI8" s="16"/>
-      <c r="AJ8" s="16"/>
-      <c r="AK8" s="16"/>
-      <c r="AL8" s="16"/>
-      <c r="AM8" s="16"/>
-      <c r="AN8" s="16"/>
-      <c r="AO8" s="16"/>
-      <c r="AP8" s="16"/>
-      <c r="AQ8" s="16"/>
-      <c r="AR8" s="16"/>
-      <c r="AS8" s="16"/>
-      <c r="AT8" s="16"/>
-      <c r="AU8" s="16"/>
-      <c r="AV8" s="16"/>
-      <c r="AW8" s="16"/>
-      <c r="AX8" s="16"/>
-      <c r="AY8" s="16"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="61"/>
+      <c r="M8" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="N8" s="61"/>
+      <c r="O8" s="61"/>
+      <c r="P8" s="63">
+        <v>3.0</v>
+      </c>
+      <c r="Q8" s="61"/>
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
+      <c r="T8" s="61"/>
+      <c r="U8" s="61"/>
+      <c r="V8" s="61"/>
+      <c r="W8" s="65"/>
+      <c r="X8" s="61"/>
+      <c r="Y8" s="61"/>
+      <c r="Z8" s="61"/>
+      <c r="AA8" s="61"/>
+      <c r="AB8" s="61"/>
+      <c r="AC8" s="61"/>
+      <c r="AD8" s="61"/>
+      <c r="AE8" s="61"/>
+      <c r="AF8" s="61"/>
+      <c r="AG8" s="66"/>
+      <c r="AH8" s="61"/>
+      <c r="AI8" s="61"/>
+      <c r="AJ8" s="61"/>
+      <c r="AK8" s="61"/>
+      <c r="AL8" s="61"/>
+      <c r="AM8" s="61"/>
+      <c r="AN8" s="61"/>
+      <c r="AO8" s="61"/>
+      <c r="AP8" s="61"/>
+      <c r="AQ8" s="61"/>
+      <c r="AR8" s="61"/>
+      <c r="AS8" s="61"/>
+      <c r="AT8" s="61"/>
+      <c r="AU8" s="61"/>
+      <c r="AV8" s="61"/>
+      <c r="AW8" s="61"/>
+      <c r="AX8" s="61"/>
+      <c r="AY8" s="61"/>
       <c r="BA8" s="45">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="32" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
       <c r="D9" s="34"/>
       <c r="E9" s="34"/>
       <c r="F9" s="34"/>
-      <c r="G9" s="34">
-        <v>3.0</v>
-      </c>
+      <c r="G9" s="34"/>
       <c r="H9" s="34"/>
       <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="34">
+      <c r="J9" s="34">
+        <v>4.0</v>
+      </c>
+      <c r="K9" s="67"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="34">
         <v>1.0</v>
       </c>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
       <c r="O9" s="34"/>
-      <c r="P9" s="34"/>
+      <c r="P9" s="34">
+        <v>1.0</v>
+      </c>
       <c r="Q9" s="34"/>
       <c r="R9" s="34"/>
       <c r="S9" s="34"/>
@@ -61753,12 +61838,12 @@
       <c r="AY9" s="34"/>
       <c r="BA9" s="45">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="32" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B10" s="28"/>
       <c r="C10" s="28"/>
@@ -61766,18 +61851,16 @@
       <c r="E10" s="28"/>
       <c r="F10" s="28"/>
       <c r="G10" s="28">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="H10" s="28"/>
       <c r="I10" s="28"/>
       <c r="J10" s="28"/>
-      <c r="K10" s="59">
-        <v>2.0</v>
-      </c>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28">
+      <c r="K10" s="60"/>
+      <c r="L10" s="28">
         <v>1.0</v>
       </c>
+      <c r="M10" s="28"/>
       <c r="N10" s="28"/>
       <c r="O10" s="28"/>
       <c r="P10" s="28"/>
@@ -61823,20 +61906,22 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
       <c r="D11" s="28"/>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28">
-        <v>2.0</v>
-      </c>
+      <c r="G11" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="H11" s="28"/>
       <c r="I11" s="28"/>
       <c r="J11" s="28"/>
-      <c r="K11" s="59"/>
+      <c r="K11" s="60">
+        <v>2.0</v>
+      </c>
       <c r="L11" s="28"/>
       <c r="M11" s="28">
         <v>1.0</v>
@@ -61881,67 +61966,67 @@
       <c r="AY11" s="28"/>
       <c r="BA11" s="45">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="37" t="s">
-        <v>82</v>
-      </c>
-      <c r="B12" s="62"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="63">
+        <v>67</v>
+      </c>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34">
+        <v>2.0</v>
+      </c>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34">
         <v>1.0</v>
       </c>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="63">
-        <v>2.0</v>
-      </c>
-      <c r="N12" s="62"/>
-      <c r="O12" s="62"/>
-      <c r="P12" s="62"/>
-      <c r="Q12" s="62"/>
-      <c r="R12" s="62"/>
-      <c r="S12" s="62"/>
-      <c r="T12" s="62"/>
-      <c r="U12" s="62"/>
-      <c r="V12" s="62"/>
-      <c r="W12" s="64"/>
-      <c r="X12" s="62"/>
-      <c r="Y12" s="62"/>
-      <c r="Z12" s="62"/>
-      <c r="AA12" s="62"/>
-      <c r="AB12" s="62"/>
-      <c r="AC12" s="62"/>
-      <c r="AD12" s="62"/>
-      <c r="AE12" s="62"/>
-      <c r="AF12" s="62"/>
-      <c r="AG12" s="65"/>
-      <c r="AH12" s="62"/>
-      <c r="AI12" s="62"/>
-      <c r="AJ12" s="62"/>
-      <c r="AK12" s="62"/>
-      <c r="AL12" s="62"/>
-      <c r="AM12" s="62"/>
-      <c r="AN12" s="62"/>
-      <c r="AO12" s="62"/>
-      <c r="AP12" s="62"/>
-      <c r="AQ12" s="62"/>
-      <c r="AR12" s="62"/>
-      <c r="AS12" s="62"/>
-      <c r="AT12" s="62"/>
-      <c r="AU12" s="62"/>
-      <c r="AV12" s="62"/>
-      <c r="AW12" s="62"/>
-      <c r="AX12" s="62"/>
-      <c r="AY12" s="62"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="34"/>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="34"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="34"/>
+      <c r="U12" s="34"/>
+      <c r="V12" s="34"/>
+      <c r="W12" s="34"/>
+      <c r="X12" s="34"/>
+      <c r="Y12" s="34"/>
+      <c r="Z12" s="34"/>
+      <c r="AA12" s="34"/>
+      <c r="AB12" s="34"/>
+      <c r="AC12" s="34"/>
+      <c r="AD12" s="34"/>
+      <c r="AE12" s="34"/>
+      <c r="AF12" s="34"/>
+      <c r="AG12" s="34"/>
+      <c r="AH12" s="34"/>
+      <c r="AI12" s="34"/>
+      <c r="AJ12" s="34"/>
+      <c r="AK12" s="34"/>
+      <c r="AL12" s="34"/>
+      <c r="AM12" s="34"/>
+      <c r="AN12" s="34"/>
+      <c r="AO12" s="34"/>
+      <c r="AP12" s="34"/>
+      <c r="AQ12" s="34"/>
+      <c r="AR12" s="34"/>
+      <c r="AS12" s="34"/>
+      <c r="AT12" s="34"/>
+      <c r="AU12" s="34"/>
+      <c r="AV12" s="34"/>
+      <c r="AW12" s="34"/>
+      <c r="AX12" s="34"/>
+      <c r="AY12" s="34"/>
       <c r="BA12" s="45">
         <f t="shared" si="1"/>
         <v>3</v>
@@ -61949,7 +62034,7 @@
     </row>
     <row r="13">
       <c r="A13" s="37" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -62012,7 +62097,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -62136,7 +62221,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B16" s="28"/>
       <c r="C16" s="28"/>
@@ -62197,7 +62282,7 @@
     </row>
     <row r="17">
       <c r="A17" s="37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B17" s="28"/>
       <c r="C17" s="28">
@@ -62258,7 +62343,7 @@
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28"/>
@@ -62441,7 +62526,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28">
@@ -62563,7 +62648,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B23" s="28"/>
       <c r="C23" s="28">
@@ -62685,7 +62770,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="37" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -62744,7 +62829,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B26" s="28"/>
       <c r="C26" s="28"/>
@@ -62803,7 +62888,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
@@ -62921,7 +63006,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
@@ -63039,7 +63124,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="37" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B31" s="28"/>
       <c r="C31" s="28"/>
@@ -63098,7 +63183,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B32" s="28"/>
       <c r="C32" s="28"/>
@@ -63216,7 +63301,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B34" s="28"/>
       <c r="C34" s="28"/>
@@ -63393,7 +63478,7 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B37" s="28"/>
       <c r="C37" s="28"/>
@@ -63505,7 +63590,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B39" s="5">
         <f t="shared" ref="B39:AY39" si="2">SUM(B5:B37)</f>
@@ -63565,7 +63650,7 @@
       </c>
       <c r="P39" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q39" s="5">
         <f t="shared" si="2"/>
@@ -63709,7 +63794,7 @@
       </c>
       <c r="BA39" s="45">
         <f>SUM(B39:AZ39)</f>
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1"/>
@@ -64695,19 +64780,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="45" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
@@ -64723,16 +64808,16 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C3" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G3" s="50"/>
       <c r="H3" s="5"/>
@@ -64744,16 +64829,16 @@
         <v>2.0</v>
       </c>
       <c r="B4" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="50" t="s">
-        <v>137</v>
-      </c>
-      <c r="D4" s="50" t="s">
-        <v>135</v>
-      </c>
       <c r="E4" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G4" s="50"/>
       <c r="H4" s="5"/>
@@ -64765,16 +64850,16 @@
         <v>3.0</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G5" s="50"/>
       <c r="H5" s="5"/>
@@ -64786,16 +64871,16 @@
         <v>4.0</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E6" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G6" s="50"/>
       <c r="H6" s="5"/>
@@ -64807,27 +64892,27 @@
         <v>5.0</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D7" s="50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E7" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G7" s="50"/>
       <c r="H7" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I7" s="5"/>
       <c r="K7" s="45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="M7" s="45" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N7" s="5"/>
     </row>
@@ -64836,16 +64921,16 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D8" s="50" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E8" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G8" s="50"/>
       <c r="H8" s="5"/>
@@ -64857,30 +64942,30 @@
         <v>7.0</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D9" s="50" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E9" s="50" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G9" s="50"/>
       <c r="H9" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I9" s="5">
         <v>3.0</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N9" s="5">
         <v>4.0</v>
@@ -64891,30 +64976,30 @@
         <v>8.0</v>
       </c>
       <c r="B10" s="50" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D10" s="50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E10" s="50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G10" s="50"/>
       <c r="H10" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I10" s="5">
         <v>2.0</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N10" s="5">
         <v>2.0</v>
@@ -64925,30 +65010,30 @@
         <v>9.0</v>
       </c>
       <c r="B11" s="50" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D11" s="50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E11" s="50" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G11" s="50"/>
       <c r="H11" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I11" s="5">
         <v>2.0</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N11" s="5">
         <v>2.0</v>
@@ -64959,28 +65044,28 @@
         <v>10.0</v>
       </c>
       <c r="B12" s="50" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D12" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E12" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G12" s="50"/>
       <c r="H12" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I12" s="5"/>
       <c r="K12" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="N12" s="5">
         <v>2.0</v>
@@ -64991,29 +65076,29 @@
         <v>11.0</v>
       </c>
       <c r="B13" s="50" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D13" s="50" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E13" s="50" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F13" s="50"/>
       <c r="G13" s="50"/>
       <c r="H13" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I13" s="5"/>
       <c r="K13" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L13" s="5"/>
       <c r="M13" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="N13" s="5">
         <v>2.0</v>
@@ -65024,31 +65109,31 @@
         <v>12.0</v>
       </c>
       <c r="B14" s="50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D14" s="50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E14" s="50" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G14" s="50"/>
       <c r="H14" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I14" s="5"/>
       <c r="K14" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="N14" s="66">
-        <v>1.0</v>
+        <v>162</v>
+      </c>
+      <c r="N14" s="5">
+        <v>2.0</v>
       </c>
     </row>
     <row r="15">
@@ -65056,30 +65141,30 @@
         <v>13.0</v>
       </c>
       <c r="B15" s="50" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D15" s="50" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E15" s="50" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G15" s="50"/>
       <c r="H15" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I15" s="5"/>
       <c r="K15" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="N15" s="66">
+        <v>156</v>
+      </c>
+      <c r="N15" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65088,30 +65173,30 @@
         <v>14.0</v>
       </c>
       <c r="B16" s="50" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D16" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E16" s="50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G16" s="50"/>
       <c r="H16" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I16" s="5"/>
       <c r="K16" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="N16" s="66">
+      <c r="N16" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65119,23 +65204,27 @@
       <c r="A17" s="50">
         <v>15.0</v>
       </c>
-      <c r="B17" s="50"/>
-      <c r="C17" s="50"/>
+      <c r="B17" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>181</v>
+      </c>
       <c r="D17" s="50"/>
       <c r="E17" s="50"/>
       <c r="G17" s="50"/>
       <c r="H17" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I17" s="5"/>
       <c r="K17" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="L17" s="5"/>
       <c r="M17" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="N17" s="66">
+        <v>142</v>
+      </c>
+      <c r="N17" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65149,15 +65238,17 @@
       <c r="E18" s="50"/>
       <c r="G18" s="50"/>
       <c r="H18" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I18" s="5"/>
-      <c r="K18" s="5"/>
+      <c r="K18" s="5" t="s">
+        <v>183</v>
+      </c>
       <c r="L18" s="5"/>
       <c r="M18" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="N18" s="66">
+        <v>165</v>
+      </c>
+      <c r="N18" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65170,14 +65261,16 @@
       <c r="D19" s="50"/>
       <c r="E19" s="50"/>
       <c r="G19" s="50"/>
-      <c r="H19" s="5"/>
+      <c r="H19" s="5" t="s">
+        <v>184</v>
+      </c>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="N19" s="66">
+        <v>159</v>
+      </c>
+      <c r="N19" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65190,14 +65283,16 @@
       <c r="D20" s="50"/>
       <c r="E20" s="50"/>
       <c r="G20" s="50"/>
-      <c r="H20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>162</v>
+      </c>
       <c r="I20" s="5"/>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="N20" s="66">
+        <v>173</v>
+      </c>
+      <c r="N20" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65210,14 +65305,14 @@
       <c r="D21" s="50"/>
       <c r="E21" s="50"/>
       <c r="G21" s="50"/>
-      <c r="H21" s="67"/>
+      <c r="H21" s="69"/>
       <c r="I21" s="5"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="N21" s="66">
+        <v>185</v>
+      </c>
+      <c r="N21" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65235,9 +65330,9 @@
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="N22" s="66">
+        <v>176</v>
+      </c>
+      <c r="N22" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65255,9 +65350,9 @@
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="N23" s="66">
+        <v>169</v>
+      </c>
+      <c r="N23" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65270,14 +65365,14 @@
       <c r="D24" s="50"/>
       <c r="E24" s="50"/>
       <c r="G24" s="50"/>
-      <c r="H24" s="67"/>
+      <c r="H24" s="69"/>
       <c r="I24" s="5"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="N24" s="66">
+        <v>179</v>
+      </c>
+      <c r="N24" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65295,9 +65390,9 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="N25" s="66">
+        <v>172</v>
+      </c>
+      <c r="N25" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65315,9 +65410,9 @@
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="N26" s="66">
+        <v>182</v>
+      </c>
+      <c r="N26" s="68">
         <v>1.0</v>
       </c>
     </row>
@@ -65333,8 +65428,12 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="K27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
+      <c r="M27" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="N27" s="68">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="50">
@@ -65348,8 +65447,12 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
       <c r="K28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
+      <c r="M28" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="N28" s="68">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="50">

</xml_diff>